<commit_message>
feat: Persistente Timer, grüne Completion-Markierung, Set-Nummerierung entfernt
- Timer mit localStorage und Timestamps für Persistenz über Tab-Wechsel/Browser-Schließen
- Übungen werden grün markiert wenn alle Sätze geloggt sind
- Set-Nummerierung (Satz X) in allen Views entfernt
- Production Migration Guide hinzugefügt
</commit_message>
<xml_diff>
--- a/Exercises.xlsx
+++ b/Exercises.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1k0/Projects/Workout-Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A00607EA-D8B6-9C44-B311-AC54935593BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA53650-BCFE-244F-A42F-E88A0040B12C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
   </bookViews>
@@ -830,6 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -861,7 +862,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -884,7 +885,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -907,7 +908,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -930,7 +931,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -953,7 +954,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -976,7 +977,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -999,7 +1000,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1022,7 +1023,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1068,7 +1069,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1091,7 +1092,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1114,7 +1115,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1137,7 +1138,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1160,7 +1161,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1183,7 +1184,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1229,7 +1230,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1252,7 +1253,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1275,7 +1276,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1298,7 +1299,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1321,7 +1322,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1344,7 +1345,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1367,7 +1368,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1390,7 +1391,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1413,7 +1414,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1436,7 +1437,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1459,7 +1460,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1505,7 +1506,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1528,7 +1529,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1551,7 +1552,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1574,7 +1575,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1620,7 +1621,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1643,7 +1644,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1827,7 +1828,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1850,7 +1851,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1873,7 +1874,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1896,7 +1897,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1919,7 +1920,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1942,7 +1943,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1965,7 +1966,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1988,7 +1989,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2011,7 +2012,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2034,7 +2035,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2080,7 +2081,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2103,7 +2104,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2126,7 +2127,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2149,7 +2150,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2172,7 +2173,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2195,7 +2196,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2218,7 +2219,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2241,7 +2242,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2264,7 +2265,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2287,7 +2288,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2310,7 +2311,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2333,7 +2334,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2356,7 +2357,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2379,7 +2380,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2402,7 +2403,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2448,7 +2449,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2471,7 +2472,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2494,7 +2495,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2540,7 +2541,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2563,7 +2564,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2586,7 +2587,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2609,7 +2610,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2632,7 +2633,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2655,7 +2656,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2678,7 +2679,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2701,7 +2702,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2724,7 +2725,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2747,7 +2748,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2770,7 +2771,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2793,7 +2794,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2816,7 +2817,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2839,7 +2840,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2862,7 +2863,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2885,7 +2886,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2908,7 +2909,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2931,7 +2932,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2954,7 +2955,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2977,7 +2978,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3000,7 +3001,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3023,7 +3024,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3046,7 +3047,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3069,7 +3070,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3092,7 +3093,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3115,7 +3116,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3138,7 +3139,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3161,7 +3162,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3184,7 +3185,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3207,7 +3208,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3230,7 +3231,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3253,7 +3254,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3276,7 +3277,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3299,7 +3300,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3322,7 +3323,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3345,7 +3346,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3368,7 +3369,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3391,7 +3392,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3437,7 +3438,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3483,7 +3484,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3506,7 +3507,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3529,7 +3530,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3553,7 +3554,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:G118" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}"/>
+  <autoFilter ref="B1:G118" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Kurzhantel"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="ja"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Add CSV ID to exercises for reliable matching
- Add csvId field to Exercise schema (unique, nullable)
- Create Prisma migration for csvId column
- Add assign-csv-ids.ts script to assign CSV IDs to exercises
- Update update-exercises.ts to match by csvId first, then by name
- Add verify-exercises.ts for exercise database verification
- Add fix-exercises.ts to fix name mismatches in production
- Update Exercises.csv (remove unused exercises)
- Remove Kurzhantel/Langhantel Skull Crushers from CSV
</commit_message>
<xml_diff>
--- a/Exercises.xlsx
+++ b/Exercises.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1k0/Projects/Workout-Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B300AA6-FFA3-B54B-8A0E-EDA2AB6E7569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71480F7-1E2F-3449-974E-861E4E048B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$B$1:$G$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$B$1:$G$116</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="138">
   <si>
     <t>Equipment</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Kurzhantel Shrug</t>
   </si>
   <si>
-    <t>Kurzhantel Skull Crushers</t>
-  </si>
-  <si>
     <t>Langhantel</t>
   </si>
   <si>
@@ -435,9 +432,6 @@
   </si>
   <si>
     <t>Kurzhantel Überkopf Extension</t>
-  </si>
-  <si>
-    <t>Langhantel Skull Crushers</t>
   </si>
   <si>
     <t>Gewicht 2x</t>
@@ -830,7 +824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34.33203125" bestFit="1" customWidth="1"/>
@@ -840,25 +834,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" t="s">
         <v>124</v>
       </c>
-      <c r="F1" t="s">
-        <v>125</v>
-      </c>
       <c r="G1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -866,22 +860,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" t="s">
-        <v>59</v>
-      </c>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -892,19 +886,19 @@
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
         <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -912,22 +906,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -935,22 +929,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -958,22 +952,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -981,22 +975,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -1004,22 +998,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1027,22 +1021,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1050,22 +1044,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s">
         <v>23</v>
       </c>
       <c r="E10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1073,22 +1067,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1096,22 +1090,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1119,22 +1113,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1142,22 +1136,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1165,22 +1159,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1188,22 +1182,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1211,22 +1205,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1234,22 +1228,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1257,22 +1251,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1280,22 +1274,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1303,22 +1297,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1326,22 +1320,22 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1349,22 +1343,22 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1375,19 +1369,19 @@
         <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1398,19 +1392,19 @@
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D25" t="s">
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1418,22 +1412,22 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F26" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1441,22 +1435,22 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1467,19 +1461,19 @@
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1487,22 +1481,22 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1513,19 +1507,19 @@
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D30" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1536,19 +1530,19 @@
         <v>25</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D31" t="s">
         <v>23</v>
       </c>
       <c r="E31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1559,19 +1553,19 @@
         <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1579,22 +1573,22 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D33" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G33" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1605,19 +1599,19 @@
         <v>21</v>
       </c>
       <c r="C34" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1625,22 +1619,22 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" t="s">
         <v>77</v>
       </c>
-      <c r="C35" t="s">
-        <v>78</v>
-      </c>
       <c r="D35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1651,19 +1645,19 @@
         <v>7</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D36" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1671,22 +1665,22 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1694,22 +1688,22 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D38" t="s">
         <v>23</v>
       </c>
       <c r="E38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1720,19 +1714,19 @@
         <v>26</v>
       </c>
       <c r="C39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D39" t="s">
         <v>23</v>
       </c>
       <c r="E39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1740,22 +1734,22 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D40" t="s">
         <v>23</v>
       </c>
       <c r="E40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1766,19 +1760,19 @@
         <v>8</v>
       </c>
       <c r="C41" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D41" t="s">
         <v>23</v>
       </c>
       <c r="E41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F41" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G41" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1789,19 +1783,19 @@
         <v>27</v>
       </c>
       <c r="C42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D42" t="s">
         <v>23</v>
       </c>
       <c r="E42" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1812,19 +1806,19 @@
         <v>28</v>
       </c>
       <c r="C43" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D43" t="s">
         <v>23</v>
       </c>
       <c r="E43" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F43" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G43" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1832,22 +1826,22 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C44" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F44" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1855,22 +1849,22 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C45" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D45" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E45" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G45" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1878,22 +1872,22 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C46" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F46" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1904,19 +1898,19 @@
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
       </c>
       <c r="E47" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G47" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1927,19 +1921,19 @@
         <v>11</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
       </c>
       <c r="E48" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F48" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G48" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1947,22 +1941,22 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C49" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1970,22 +1964,22 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C50" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1993,22 +1987,22 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C51" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D51" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E51" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F51" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G51" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -2016,22 +2010,22 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C52" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D52" t="s">
         <v>23</v>
       </c>
       <c r="E52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -2039,22 +2033,22 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D53" t="s">
         <v>23</v>
       </c>
       <c r="E53" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F53" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G53" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -2065,19 +2059,19 @@
         <v>29</v>
       </c>
       <c r="C54" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D54" t="s">
         <v>23</v>
       </c>
       <c r="E54" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -2085,22 +2079,22 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C55" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D55" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E55" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G55" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -2108,22 +2102,22 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D56" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E56" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F56" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G56" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -2134,19 +2128,19 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D57" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E57" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F57" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G57" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -2154,22 +2148,22 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D58" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E58" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F58" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G58" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -2177,22 +2171,22 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D59" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E59" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G59" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -2200,22 +2194,22 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D60" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E60" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F60" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G60" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -2223,22 +2217,22 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C61" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D61" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E61" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F61" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G61" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -2246,22 +2240,22 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D62" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E62" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F62" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G62" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -2269,22 +2263,22 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C63" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D63" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E63" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F63" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G63" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2292,22 +2286,22 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C64" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D64" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E64" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G64" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
@@ -2318,19 +2312,19 @@
         <v>14</v>
       </c>
       <c r="C65" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D65" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F65" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2338,22 +2332,22 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C66" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D66" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E66" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F66" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G66" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2361,22 +2355,22 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C67" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D67" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E67" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F67" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G67" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2384,22 +2378,22 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C68" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D68" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E68" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F68" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G68" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -2407,22 +2401,22 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C69" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D69" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E69" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F69" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G69" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2433,19 +2427,19 @@
         <v>30</v>
       </c>
       <c r="C70" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D70" t="s">
         <v>23</v>
       </c>
       <c r="E70" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F70" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G70" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2456,19 +2450,19 @@
         <v>15</v>
       </c>
       <c r="C71" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D71" t="s">
         <v>23</v>
       </c>
       <c r="E71" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F71" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G71" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2479,19 +2473,19 @@
         <v>16</v>
       </c>
       <c r="C72" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D72" t="s">
         <v>23</v>
       </c>
       <c r="E72" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G72" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2499,22 +2493,22 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C73" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D73" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E73" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F73" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G73" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -2525,19 +2519,19 @@
         <v>31</v>
       </c>
       <c r="C74" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D74" t="s">
         <v>23</v>
       </c>
       <c r="E74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F74" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -2545,22 +2539,22 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D75" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E75" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F75" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G75" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -2568,22 +2562,22 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C76" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D76" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E76" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F76" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G76" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
@@ -2591,22 +2585,22 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C77" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D77" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E77" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F77" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G77" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
@@ -2614,22 +2608,22 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C78" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D78" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E78" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G78" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2640,19 +2634,19 @@
         <v>17</v>
       </c>
       <c r="C79" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D79" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E79" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F79" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G79" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -2660,22 +2654,22 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C80" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D80" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E80" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F80" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G80" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -2683,22 +2677,22 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C81" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D81" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E81" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G81" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -2709,19 +2703,19 @@
         <v>18</v>
       </c>
       <c r="C82" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D82" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E82" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F82" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G82" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
@@ -2732,19 +2726,19 @@
         <v>19</v>
       </c>
       <c r="C83" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D83" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E83" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F83" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G83" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
@@ -2752,22 +2746,22 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C84" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D84" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E84" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F84" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G84" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
@@ -2775,22 +2769,22 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C85" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D85" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E85" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G85" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
@@ -2798,22 +2792,22 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C86" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D86" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E86" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G86" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
@@ -2821,22 +2815,22 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C87" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D87" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E87" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F87" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G87" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -2844,22 +2838,22 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C88" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D88" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E88" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F88" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G88" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
@@ -2867,22 +2861,22 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C89" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D89" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F89" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -2890,22 +2884,22 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C90" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D90" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E90" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F90" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G90" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
@@ -2913,22 +2907,22 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C91" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D91" t="s">
         <v>23</v>
       </c>
       <c r="E91" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
@@ -2936,22 +2930,22 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C92" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D92" t="s">
         <v>23</v>
       </c>
       <c r="E92" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
@@ -2959,22 +2953,22 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C93" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D93" t="s">
         <v>23</v>
       </c>
       <c r="E93" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F93" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G93" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
@@ -2985,19 +2979,19 @@
         <v>5</v>
       </c>
       <c r="C94" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D94" t="s">
         <v>23</v>
       </c>
       <c r="E94" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G94" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
@@ -3008,19 +3002,19 @@
         <v>6</v>
       </c>
       <c r="C95" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D95" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E95" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F95" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G95" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
@@ -3028,22 +3022,22 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C96" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D96" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E96" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F96" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G96" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
@@ -3051,22 +3045,22 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C97" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D97" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E97" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F97" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G97" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
@@ -3074,22 +3068,22 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C98" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D98" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E98" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F98" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G98" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
@@ -3097,22 +3091,22 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C99" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D99" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E99" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G99" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
@@ -3120,22 +3114,22 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C100" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D100" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E100" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G100" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
@@ -3146,19 +3140,19 @@
         <v>32</v>
       </c>
       <c r="C101" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D101" t="s">
         <v>23</v>
       </c>
       <c r="E101" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F101" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G101" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
@@ -3166,22 +3160,22 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C102" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D102" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E102" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F102" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G102" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
@@ -3189,22 +3183,22 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C103" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D103" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E103" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F103" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G103" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
@@ -3212,22 +3206,22 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C104" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D104" t="s">
         <v>23</v>
       </c>
       <c r="E104" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F104" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G104" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -3235,22 +3229,22 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C105" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D105" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E105" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F105" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G105" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
@@ -3258,22 +3252,22 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C106" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D106" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E106" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F106" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G106" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
@@ -3281,22 +3275,22 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C107" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D107" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E107" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F107" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G107" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
@@ -3304,22 +3298,22 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C108" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D108" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E108" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F108" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G108" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
@@ -3327,22 +3321,22 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C109" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D109" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E109" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F109" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G109" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
@@ -3350,22 +3344,22 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C110" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D110" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E110" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F110" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G110" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
@@ -3376,19 +3370,19 @@
         <v>12</v>
       </c>
       <c r="C111" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D111" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E111" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F111" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G111" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -3396,22 +3390,22 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="C112" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D112" t="s">
         <v>23</v>
       </c>
       <c r="E112" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F112" t="s">
         <v>126</v>
       </c>
       <c r="G112" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.2">
@@ -3419,10 +3413,10 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>83</v>
+        <v>130</v>
       </c>
       <c r="C113" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D113" t="s">
         <v>23</v>
@@ -3431,10 +3425,10 @@
         <v>126</v>
       </c>
       <c r="F113" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G113" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.2">
@@ -3442,22 +3436,22 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="C114" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D114" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E114" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F114" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G114" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
@@ -3465,22 +3459,22 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="C115" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D115" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="E115" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F115" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G115" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.2">
@@ -3491,69 +3485,23 @@
         <v>115</v>
       </c>
       <c r="C116" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D116" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="E116" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F116" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G116" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A117">
-        <v>116</v>
-      </c>
-      <c r="B117" t="s">
-        <v>13</v>
-      </c>
-      <c r="C117" t="s">
-        <v>81</v>
-      </c>
-      <c r="D117" t="s">
-        <v>10</v>
-      </c>
-      <c r="E117" t="s">
-        <v>127</v>
-      </c>
-      <c r="F117" t="s">
-        <v>126</v>
-      </c>
-      <c r="G117" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A118">
-        <v>117</v>
-      </c>
-      <c r="B118" t="s">
-        <v>116</v>
-      </c>
-      <c r="C118" t="s">
-        <v>81</v>
-      </c>
-      <c r="D118" t="s">
-        <v>10</v>
-      </c>
-      <c r="E118" t="s">
-        <v>127</v>
-      </c>
-      <c r="F118" t="s">
-        <v>126</v>
-      </c>
-      <c r="G118" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:G118" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}"/>
+  <autoFilter ref="B1:G116" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Update deployment guide with lessons learned from 6. April production deployment
- Add pre-deployment checks (local build testing)
- Document deployment options (automatic vs manual)
- Add SSH tunnel instructions for database migrations
- Add troubleshooting sections (TypeScript, SSH tunnel, name-mismatch)
- Document CSV-ID system implementation
- Add comprehensive lessons learned from 6. April deployment
- Update exercises CSV (removed unused Skull Crusher variants, now 115 exercises)
</commit_message>
<xml_diff>
--- a/Exercises.xlsx
+++ b/Exercises.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1k0/Projects/Workout-Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71480F7-1E2F-3449-974E-861E4E048B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2A38D4-EECF-1943-8626-714694987B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -824,6 +824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -855,7 +856,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -878,7 +879,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -901,7 +902,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -924,7 +925,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -947,7 +948,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -970,7 +971,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -993,7 +994,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1030,16 +1031,16 @@
         <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G9" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1062,7 +1063,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1085,7 +1086,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1108,7 +1109,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1131,7 +1132,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1154,7 +1155,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1177,7 +1178,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1200,7 +1201,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1223,7 +1224,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1246,7 +1247,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1269,7 +1270,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1292,7 +1293,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1315,7 +1316,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1338,7 +1339,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1361,7 +1362,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1384,7 +1385,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1430,7 +1431,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1453,7 +1454,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1522,7 +1523,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1545,7 +1546,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1568,7 +1569,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1605,7 +1606,7 @@
         <v>41</v>
       </c>
       <c r="E34" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F34" t="s">
         <v>126</v>
@@ -1614,7 +1615,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1660,7 +1661,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1683,7 +1684,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1706,7 +1707,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1752,7 +1753,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1775,7 +1776,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1844,7 +1845,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1867,7 +1868,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1890,7 +1891,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1913,7 +1914,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1936,7 +1937,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1982,7 +1983,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2028,7 +2029,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2051,7 +2052,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2074,7 +2075,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2097,7 +2098,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2120,7 +2121,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2143,7 +2144,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2166,7 +2167,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2189,7 +2190,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2212,7 +2213,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2235,7 +2236,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2258,7 +2259,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2281,7 +2282,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2304,7 +2305,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2327,7 +2328,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2350,7 +2351,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2373,7 +2374,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2396,7 +2397,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2442,7 +2443,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2465,7 +2466,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2488,7 +2489,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2511,7 +2512,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2534,7 +2535,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2557,7 +2558,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2580,7 +2581,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2603,7 +2604,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2626,7 +2627,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2649,7 +2650,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2672,7 +2673,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2695,7 +2696,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2718,7 +2719,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2741,7 +2742,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2764,7 +2765,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2787,7 +2788,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2810,7 +2811,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2833,7 +2834,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2856,7 +2857,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2879,7 +2880,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2902,7 +2903,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2925,7 +2926,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2948,7 +2949,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2971,7 +2972,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2994,7 +2995,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3017,7 +3018,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3040,7 +3041,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3063,7 +3064,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3109,7 +3110,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3132,7 +3133,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3155,7 +3156,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3178,7 +3179,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3201,7 +3202,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3224,7 +3225,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3270,7 +3271,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3293,7 +3294,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3316,7 +3317,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3339,7 +3340,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3362,7 +3363,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3385,7 +3386,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3408,7 +3409,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3431,7 +3432,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3454,7 +3455,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3477,7 +3478,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3501,7 +3502,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:G116" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}"/>
+  <autoFilter ref="B1:G116" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Unilateral Butterfly Reverse"/>
+        <filter val="Unilateral Kabel Latzug"/>
+        <filter val="Unilateral Trizeps Kabel Kickbacks"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Workout Templates System
- Add WorkoutTemplate, WorkoutTemplateExercise, WorkoutTemplateSet models
- Add CSV import script with 10 system templates
- Add backend API: CRUD + from-blueprint + from-workout + start-from-template
- Rename /exercises to /templates with 2 tabs (Übungen | Workout-Vorlagen)
- Add TemplateSelectionModal (reusable)
- Add template loading in cycle wizard (Aus Vorlage wählen)
- Add template creation from blueprints and completed workouts
- Add template editor as full-screen page (Past-Workout style)
- Fix plannedSets display (order vs setNumber mapping)
- Fix template save modal persistence (WorkoutContext)
- Fix set order conversion in cycle wizard (0-based to 1-based)

Database changes:
- New migration: 20260406214642_add_workout_templates
- Includes CSV import: 10 system workout templates (German)
- Supports custom user templates with CRUD operations
</commit_message>
<xml_diff>
--- a/Exercises.xlsx
+++ b/Exercises.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1k0/Projects/Workout-Tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2A38D4-EECF-1943-8626-714694987B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCDA4CDA-6902-8D4F-B4F2-0378BA9A64DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{B03716CD-46A2-6341-9F01-26B207CBC3B3}"/>
   </bookViews>
@@ -824,7 +824,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -856,7 +855,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -879,7 +878,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -902,7 +901,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -925,7 +924,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -948,7 +947,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -971,7 +970,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -994,7 +993,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1040,7 +1039,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1063,7 +1062,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1086,7 +1085,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1109,7 +1108,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1132,7 +1131,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1155,7 +1154,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1178,7 +1177,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1201,7 +1200,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1224,7 +1223,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1247,7 +1246,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1270,7 +1269,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1316,7 +1315,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1339,7 +1338,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1362,7 +1361,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1385,7 +1384,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1408,7 +1407,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1431,7 +1430,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1454,7 +1453,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1477,7 +1476,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1500,7 +1499,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1523,7 +1522,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1546,7 +1545,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1569,7 +1568,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1615,7 +1614,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1638,7 +1637,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1661,7 +1660,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1684,7 +1683,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1707,7 +1706,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1730,7 +1729,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1753,7 +1752,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1776,7 +1775,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1799,7 +1798,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1822,7 +1821,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1845,7 +1844,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1868,7 +1867,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1891,7 +1890,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1914,7 +1913,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1937,7 +1936,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1960,7 +1959,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1983,7 +1982,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2006,7 +2005,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2029,7 +2028,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2052,7 +2051,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2075,7 +2074,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2098,7 +2097,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2121,7 +2120,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2144,7 +2143,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2167,7 +2166,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2190,7 +2189,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2213,7 +2212,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2236,7 +2235,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2259,7 +2258,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2282,7 +2281,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2305,7 +2304,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2328,7 +2327,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2351,7 +2350,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2374,7 +2373,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2397,7 +2396,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2420,7 +2419,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2443,7 +2442,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2466,7 +2465,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2489,7 +2488,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2512,7 +2511,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2535,7 +2534,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2558,7 +2557,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2581,7 +2580,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2604,7 +2603,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2627,7 +2626,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2650,7 +2649,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2673,7 +2672,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2696,7 +2695,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2719,7 +2718,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2742,7 +2741,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2765,7 +2764,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2788,7 +2787,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2811,7 +2810,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2834,7 +2833,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2857,7 +2856,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2880,7 +2879,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2903,7 +2902,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2926,7 +2925,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2949,7 +2948,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2972,7 +2971,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2995,7 +2994,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3018,7 +3017,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3041,7 +3040,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3064,7 +3063,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3087,7 +3086,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3110,7 +3109,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3133,7 +3132,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3156,7 +3155,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3179,7 +3178,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3202,7 +3201,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3225,7 +3224,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3271,7 +3270,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3294,7 +3293,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3317,7 +3316,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3340,7 +3339,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3363,7 +3362,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3386,7 +3385,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3409,7 +3408,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3432,7 +3431,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3455,7 +3454,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3478,7 +3477,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3502,15 +3501,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:G116" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Unilateral Butterfly Reverse"/>
-        <filter val="Unilateral Kabel Latzug"/>
-        <filter val="Unilateral Trizeps Kabel Kickbacks"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:G116" xr:uid="{F341F40E-1D30-564C-B355-EE20718AED3C}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>